<commit_message>
Rule 2 keeps 3 AV weeks (drop wk+3); rebuild 10-23 report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_10-23.xlsx
+++ b/Stock_Daily_Reefer_10-23.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'TOTAL RH'!$A$1:$Q$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'TOTAL RH'!$A$1:$Q$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'YEAR BUILT'!$A$1:$Q$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10554,7 +10554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.571428571428571" customWidth="1" min="1" max="1"/>
@@ -10904,11 +10904,11 @@
         </is>
       </c>
       <c r="N9" s="10">
-        <f>C6+C7+C10+C13+C16</f>
+        <f>C6+C7+C10+C13</f>
         <v/>
       </c>
       <c r="O9" s="10">
-        <f>D6+D7+D10+D13+D16</f>
+        <f>D6+D7+D10+D13</f>
         <v/>
       </c>
     </row>
@@ -10955,11 +10955,11 @@
         </is>
       </c>
       <c r="N10" s="10">
-        <f>I6+I7+I10+I13+I16</f>
+        <f>I6+I7+I10+I13</f>
         <v/>
       </c>
       <c r="O10" s="10">
-        <f>J6+J7+J10+J13+J16</f>
+        <f>J6+J7+J10+J13</f>
         <v/>
       </c>
     </row>
@@ -11115,25 +11115,25 @@
         </is>
       </c>
       <c r="N14" s="10">
-        <f>C17</f>
+        <f>C14</f>
         <v/>
       </c>
       <c r="O14" s="10">
-        <f>D17</f>
+        <f>D14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="1" t="n"/>
+      <c r="D15" s="1" t="n"/>
       <c r="E15" s="1" t="n"/>
       <c r="F15" s="1" t="n"/>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
+      <c r="G15" s="1" t="n"/>
+      <c r="H15" s="1" t="n"/>
+      <c r="I15" s="1" t="n"/>
+      <c r="J15" s="1" t="n"/>
       <c r="K15" s="1" t="n"/>
       <c r="L15" s="1" t="n"/>
       <c r="M15" s="9" t="inlineStr">
@@ -11142,49 +11142,25 @@
         </is>
       </c>
       <c r="N15" s="10">
-        <f>I17</f>
+        <f>I14</f>
         <v/>
       </c>
       <c r="O15" s="10">
-        <f>J17</f>
+        <f>J14</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="14">
-        <f>Control!$A$7</f>
-        <v/>
-      </c>
-      <c r="B16" s="9">
-        <f>"Booking on "&amp;IF(Control!$B7=Control!$C7,DAY(Control!$B7)&amp;" "&amp;CHOOSE(MONTH(Control!$B7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B7)=MONTH(Control!$C7),DAY(Control!$B7)&amp;"-"&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B7)&amp;" "&amp;CHOOSE(MONTH(Control!$B7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
-        <v/>
-      </c>
-      <c r="C16" s="9">
-        <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B7,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C7)</f>
-        <v/>
-      </c>
-      <c r="D16" s="9">
-        <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"BKK27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B7,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C7)</f>
-        <v/>
-      </c>
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="1" t="n"/>
+      <c r="D16" s="1" t="n"/>
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="n"/>
-      <c r="G16" s="14">
-        <f>Control!$A$7</f>
-        <v/>
-      </c>
-      <c r="H16" s="9">
-        <f>"Booking on "&amp;IF(Control!$B7=Control!$C7,DAY(Control!$B7)&amp;" "&amp;CHOOSE(MONTH(Control!$B7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),IF(MONTH(Control!$B7)=MONTH(Control!$C7),DAY(Control!$B7)&amp;"-"&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"),DAY(Control!$B7)&amp;" "&amp;CHOOSE(MONTH(Control!$B7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")&amp;"-"&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")))</f>
-        <v/>
-      </c>
-      <c r="I16" s="9">
-        <f>SUMIFS(BookingRaw!$C$2:$C$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B7,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C7)</f>
-        <v/>
-      </c>
-      <c r="J16" s="9">
-        <f>SUMIFS(BookingRaw!$D$2:$D$8000,BookingRaw!$A$2:$A$8000,"LCH27",BookingRaw!$B$2:$B$8000,"&gt;="&amp;Control!$B7,BookingRaw!$B$2:$B$8000,"&lt;="&amp;Control!$C7)</f>
-        <v/>
-      </c>
+      <c r="G16" s="1" t="n"/>
+      <c r="H16" s="1" t="n"/>
+      <c r="I16" s="1" t="n"/>
+      <c r="J16" s="1" t="n"/>
       <c r="K16" s="1" t="n"/>
       <c r="L16" s="1" t="n"/>
       <c r="M16" s="15" t="inlineStr">
@@ -11202,33 +11178,39 @@
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="16">
-        <f>"AV Balance till "&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
-        <v/>
-      </c>
-      <c r="C17" s="59">
-        <f>C14-C16</f>
-        <v/>
-      </c>
-      <c r="D17" s="60">
-        <f>D14-D16</f>
-        <v/>
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>BKK27 / BC2</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
       </c>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="16">
-        <f>"AV Balance till "&amp;DAY(Control!$C7)&amp;" "&amp;CHOOSE(MONTH(Control!$C7),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
-        <v/>
-      </c>
-      <c r="I17" s="59">
-        <f>I14-I16</f>
-        <v/>
-      </c>
-      <c r="J17" s="59">
-        <f>J14-J16</f>
-        <v/>
+      <c r="G17" s="1" t="n"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>LCH27 / HAST</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
       </c>
       <c r="K17" s="1" t="n"/>
       <c r="L17" s="1" t="n"/>
@@ -11238,15 +11220,35 @@
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IER")</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IER")</f>
+        <v/>
+      </c>
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="n"/>
       <c r="G18" s="1" t="n"/>
-      <c r="H18" s="1" t="n"/>
-      <c r="I18" s="1" t="n"/>
-      <c r="J18" s="1" t="n"/>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="I18" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IER")</f>
+        <v/>
+      </c>
+      <c r="J18" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IER")</f>
+        <v/>
+      </c>
       <c r="K18" s="1" t="n"/>
       <c r="L18" s="1" t="n"/>
       <c r="M18" s="1" t="n"/>
@@ -11255,15 +11257,35 @@
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="1" t="n"/>
-      <c r="B19" s="1" t="n"/>
-      <c r="C19" s="1" t="n"/>
-      <c r="D19" s="1" t="n"/>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"OER")</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"OER")</f>
+        <v/>
+      </c>
       <c r="E19" s="1" t="n"/>
       <c r="F19" s="1" t="n"/>
       <c r="G19" s="1" t="n"/>
-      <c r="H19" s="1" t="n"/>
-      <c r="I19" s="1" t="n"/>
-      <c r="J19" s="1" t="n"/>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="I19" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"OER")</f>
+        <v/>
+      </c>
+      <c r="J19" s="10">
+        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"OER")</f>
+        <v/>
+      </c>
       <c r="K19" s="1" t="n"/>
       <c r="L19" s="1" t="n"/>
       <c r="M19" s="1" t="n"/>
@@ -11272,39 +11294,15 @@
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="1" t="n"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>BKK27 / BC2</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
       <c r="E20" s="1" t="n"/>
       <c r="F20" s="1" t="n"/>
       <c r="G20" s="1" t="n"/>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>LCH27 / HAST</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
       <c r="K20" s="1" t="n"/>
       <c r="L20" s="1" t="n"/>
       <c r="M20" s="1" t="n"/>
@@ -11313,35 +11311,15 @@
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="1" t="n"/>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>AV</t>
-        </is>
-      </c>
-      <c r="C21" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IER")</f>
-        <v/>
-      </c>
-      <c r="D21" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IER")</f>
-        <v/>
-      </c>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="n"/>
       <c r="E21" s="1" t="n"/>
       <c r="F21" s="1" t="n"/>
       <c r="G21" s="1" t="n"/>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>AV</t>
-        </is>
-      </c>
-      <c r="I21" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"IER")</f>
-        <v/>
-      </c>
-      <c r="J21" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IED")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IEP")+COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"IER")</f>
-        <v/>
-      </c>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
       <c r="K21" s="1" t="n"/>
       <c r="L21" s="1" t="n"/>
       <c r="M21" s="1" t="n"/>
@@ -11350,36 +11328,24 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>DMG</t>
-        </is>
-      </c>
-      <c r="C22" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"OER")</f>
-        <v/>
-      </c>
-      <c r="D22" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"BKK27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"OER")</f>
-        <v/>
-      </c>
-      <c r="E22" s="1" t="n"/>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>BKK / BC2 (BKK27)</t>
+        </is>
+      </c>
+      <c r="C22" s="57" t="n"/>
+      <c r="D22" s="57" t="n"/>
+      <c r="E22" s="58" t="n"/>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>DMG</t>
-        </is>
-      </c>
-      <c r="I22" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"22RE",StockRaw!$C$2:$C$109,"OER")</f>
-        <v/>
-      </c>
-      <c r="J22" s="10">
-        <f>COUNTIFS(StockRaw!$A$2:$A$109,"LCH27",StockRaw!$B$2:$B$109,"45RE",StockRaw!$C$2:$C$109,"OER")</f>
-        <v/>
-      </c>
-      <c r="K22" s="1" t="n"/>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>LCH / HAST (LCH27)</t>
+        </is>
+      </c>
+      <c r="I22" s="57" t="n"/>
+      <c r="J22" s="57" t="n"/>
+      <c r="K22" s="58" t="n"/>
       <c r="L22" s="1" t="n"/>
       <c r="M22" s="1" t="n"/>
       <c r="N22" s="1" t="n"/>
@@ -11387,16 +11353,50 @@
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="1" t="n"/>
-      <c r="C23" s="1" t="n"/>
-      <c r="D23" s="1" t="n"/>
-      <c r="E23" s="1" t="n"/>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>YEAR BUILT 5 YEARS
+FOR DURIAN SEASON</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
-      <c r="H23" s="1" t="n"/>
-      <c r="I23" s="1" t="n"/>
-      <c r="J23" s="1" t="n"/>
-      <c r="K23" s="1" t="n"/>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>YEAR BUILT 5 YEARS
+FOR DURIAN SEASON</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
       <c r="N23" s="1" t="n"/>
@@ -11404,16 +11404,40 @@
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
-      <c r="E24" s="1" t="n"/>
+      <c r="B24" s="61" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
-      <c r="J24" s="1" t="n"/>
-      <c r="K24" s="1" t="n"/>
+      <c r="H24" s="61" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
       <c r="L24" s="1" t="n"/>
       <c r="M24" s="1" t="n"/>
       <c r="N24" s="1" t="n"/>
@@ -11421,24 +11445,32 @@
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>BKK / BC2 (BKK27)</t>
-        </is>
-      </c>
-      <c r="C25" s="57" t="n"/>
-      <c r="D25" s="57" t="n"/>
-      <c r="E25" s="58" t="n"/>
+      <c r="B25" s="10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
-      <c r="H25" s="18" t="inlineStr">
-        <is>
-          <t>LCH / HAST (LCH27)</t>
-        </is>
-      </c>
-      <c r="I25" s="57" t="n"/>
-      <c r="J25" s="57" t="n"/>
-      <c r="K25" s="58" t="n"/>
+      <c r="H25" s="10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="L25" s="1" t="n"/>
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
@@ -11446,49 +11478,31 @@
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>YEAR BUILT 5 YEARS
-FOR DURIAN SEASON</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
+      <c r="B26" s="10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>YEAR BUILT 5 YEARS
-FOR DURIAN SEASON</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
+      <c r="H26" s="10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I26" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="L26" s="1" t="n"/>
       <c r="M26" s="1" t="n"/>
@@ -11497,39 +11511,31 @@
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="61" t="n"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
+      <c r="B27" s="10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
-      <c r="H27" s="61" t="n"/>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
+      <c r="H27" s="10" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n"/>
@@ -11539,7 +11545,7 @@
     <row r="28" ht="13" customHeight="1">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="10" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>0</v>
@@ -11553,7 +11559,7 @@
       <c r="F28" s="1" t="n"/>
       <c r="G28" s="1" t="n"/>
       <c r="H28" s="10" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>0</v>
@@ -11572,24 +11578,24 @@
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="10" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D29" s="10" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" s="1" t="n"/>
       <c r="G29" s="1" t="n"/>
       <c r="H29" s="10" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="I29" s="10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>0</v>
@@ -11605,10 +11611,10 @@
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="1" t="n"/>
       <c r="B30" s="10" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>0</v>
@@ -11619,10 +11625,10 @@
       <c r="F30" s="1" t="n"/>
       <c r="G30" s="1" t="n"/>
       <c r="H30" s="10" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>0</v>
@@ -11637,30 +11643,34 @@
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="10" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>0</v>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="F31" s="1" t="n"/>
       <c r="G31" s="1" t="n"/>
-      <c r="H31" s="10" t="n">
-        <v>2023</v>
-      </c>
-      <c r="I31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="10" t="n">
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="1" t="n"/>
@@ -11670,145 +11680,42 @@
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="10" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="10" t="n">
-        <v>0</v>
+      <c r="B32" s="1" t="n"/>
+      <c r="C32" s="1" t="n"/>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>OVER 5 Y</t>
+        </is>
+      </c>
+      <c r="E32" s="21" t="n">
+        <v>5</v>
       </c>
       <c r="F32" s="1" t="n"/>
       <c r="G32" s="1" t="n"/>
-      <c r="H32" s="10" t="n">
-        <v>2022</v>
-      </c>
-      <c r="I32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="10" t="n">
-        <v>0</v>
+      <c r="H32" s="1" t="n"/>
+      <c r="I32" s="1" t="n"/>
+      <c r="J32" s="20" t="inlineStr">
+        <is>
+          <t>OVER 5 Y</t>
+        </is>
+      </c>
+      <c r="K32" s="21" t="n">
+        <v>34</v>
       </c>
       <c r="L32" s="1" t="n"/>
       <c r="M32" s="1" t="n"/>
       <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
     </row>
-    <row r="33" ht="13" customHeight="1">
-      <c r="A33" s="1" t="n"/>
-      <c r="B33" s="10" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C33" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="1" t="n"/>
-      <c r="G33" s="1" t="n"/>
-      <c r="H33" s="10" t="n">
-        <v>2021</v>
-      </c>
-      <c r="I33" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" s="1" t="n"/>
-      <c r="M33" s="1" t="n"/>
-      <c r="N33" s="1" t="n"/>
-      <c r="O33" s="1" t="n"/>
-    </row>
-    <row r="34" ht="13" customHeight="1">
-      <c r="A34" s="1" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="1" t="n"/>
-      <c r="G34" s="1" t="n"/>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="J34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="1" t="n"/>
-      <c r="M34" s="1" t="n"/>
-      <c r="N34" s="1" t="n"/>
-      <c r="O34" s="1" t="n"/>
-    </row>
-    <row r="35" ht="13" customHeight="1">
-      <c r="A35" s="1" t="n"/>
-      <c r="B35" s="1" t="n"/>
-      <c r="C35" s="1" t="n"/>
-      <c r="D35" s="20" t="inlineStr">
-        <is>
-          <t>OVER 5 Y</t>
-        </is>
-      </c>
-      <c r="E35" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="F35" s="1" t="n"/>
-      <c r="G35" s="1" t="n"/>
-      <c r="H35" s="1" t="n"/>
-      <c r="I35" s="1" t="n"/>
-      <c r="J35" s="20" t="inlineStr">
-        <is>
-          <t>OVER 5 Y</t>
-        </is>
-      </c>
-      <c r="K35" s="21" t="n">
-        <v>34</v>
-      </c>
-      <c r="L35" s="1" t="n"/>
-      <c r="M35" s="1" t="n"/>
-      <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="H22:K22"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="H23:H24"/>
     <mergeCell ref="H3:J3"/>
-    <mergeCell ref="B26:B27"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="B22:E22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -12681,7 +12588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -12764,7 +12671,7 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="41">
-        <f>MIN('TOTAL RH'!D17,'TOTAL RH'!J17)</f>
+        <f>MIN('TOTAL RH'!D14,'TOTAL RH'!J14)</f>
         <v/>
       </c>
       <c r="C5" s="24" t="n"/>
@@ -12791,7 +12698,7 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="1" t="n"/>
       <c r="B6" s="43">
-        <f>"BKK27/LCH27 40'RH, worse "&amp;'TOTAL RH'!B17</f>
+        <f>"BKK27/LCH27 40'RH, worse "&amp;'TOTAL RH'!B14</f>
         <v/>
       </c>
       <c r="C6" s="24" t="n"/>
@@ -13259,33 +13166,15 @@
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
-      <c r="B22" s="50">
-        <f>'TOTAL RH'!B16</f>
-        <v/>
-      </c>
-      <c r="C22" s="51">
-        <f>'TOTAL RH'!C16</f>
-        <v/>
-      </c>
-      <c r="D22" s="51">
-        <f>'TOTAL RH'!D16</f>
-        <v/>
-      </c>
+      <c r="B22" s="1" t="n"/>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
       <c r="E22" s="1" t="n"/>
       <c r="F22" s="1" t="n"/>
       <c r="G22" s="1" t="n"/>
-      <c r="H22" s="50">
-        <f>'TOTAL RH'!H16</f>
-        <v/>
-      </c>
-      <c r="I22" s="51">
-        <f>'TOTAL RH'!I16</f>
-        <v/>
-      </c>
-      <c r="J22" s="51">
-        <f>'TOTAL RH'!J16</f>
-        <v/>
-      </c>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
       <c r="K22" s="1" t="n"/>
       <c r="L22" s="1" t="n"/>
       <c r="M22" s="1" t="n"/>
@@ -13295,33 +13184,19 @@
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
-      <c r="B23" s="52">
-        <f>'TOTAL RH'!B17</f>
-        <v/>
-      </c>
-      <c r="C23" s="53">
-        <f>'TOTAL RH'!C17</f>
-        <v/>
-      </c>
-      <c r="D23" s="64">
-        <f>'TOTAL RH'!D17</f>
-        <v/>
-      </c>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>REMARKS  (AV = move code IED/IEP/IER, DMG = move code OER)</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="n"/>
+      <c r="D23" s="1" t="n"/>
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
-      <c r="H23" s="52">
-        <f>'TOTAL RH'!H17</f>
-        <v/>
-      </c>
-      <c r="I23" s="53">
-        <f>'TOTAL RH'!I17</f>
-        <v/>
-      </c>
-      <c r="J23" s="53">
-        <f>'TOTAL RH'!J17</f>
-        <v/>
-      </c>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="1" t="n"/>
+      <c r="J23" s="1" t="n"/>
       <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
@@ -13331,15 +13206,21 @@
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
+      <c r="B24" s="45">
+        <f>'TOTAL RH'!B3</f>
+        <v/>
+      </c>
+      <c r="C24" s="62" t="n"/>
+      <c r="D24" s="63" t="n"/>
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
-      <c r="J24" s="1" t="n"/>
+      <c r="H24" s="46">
+        <f>'TOTAL RH'!H3</f>
+        <v/>
+      </c>
+      <c r="I24" s="62" t="n"/>
+      <c r="J24" s="63" t="n"/>
       <c r="K24" s="1" t="n"/>
       <c r="L24" s="1" t="n"/>
       <c r="M24" s="1" t="n"/>
@@ -13349,15 +13230,31 @@
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="1" t="n"/>
-      <c r="C25" s="1" t="n"/>
-      <c r="D25" s="1" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="47" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="D25" s="47" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
-      <c r="I25" s="1" t="n"/>
-      <c r="J25" s="1" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="47" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="J25" s="47" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
       <c r="K25" s="1" t="n"/>
       <c r="L25" s="1" t="n"/>
       <c r="M25" s="1" t="n"/>
@@ -13367,19 +13264,35 @@
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="44" t="inlineStr">
-        <is>
-          <t>REMARKS  (AV = move code IED/IEP/IER, DMG = move code OER)</t>
-        </is>
-      </c>
-      <c r="C26" s="1" t="n"/>
-      <c r="D26" s="1" t="n"/>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="C26" s="51">
+        <f>'TOTAL RH'!C18</f>
+        <v/>
+      </c>
+      <c r="D26" s="51">
+        <f>'TOTAL RH'!D18</f>
+        <v/>
+      </c>
       <c r="E26" s="1" t="n"/>
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
-      <c r="H26" s="1" t="n"/>
-      <c r="I26" s="1" t="n"/>
-      <c r="J26" s="1" t="n"/>
+      <c r="H26" s="24" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="I26" s="51">
+        <f>'TOTAL RH'!I18</f>
+        <v/>
+      </c>
+      <c r="J26" s="51">
+        <f>'TOTAL RH'!J18</f>
+        <v/>
+      </c>
       <c r="K26" s="1" t="n"/>
       <c r="L26" s="1" t="n"/>
       <c r="M26" s="1" t="n"/>
@@ -13389,21 +13302,35 @@
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="45">
-        <f>'TOTAL RH'!B3</f>
-        <v/>
-      </c>
-      <c r="C27" s="62" t="n"/>
-      <c r="D27" s="63" t="n"/>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="C27" s="51">
+        <f>'TOTAL RH'!C19</f>
+        <v/>
+      </c>
+      <c r="D27" s="51">
+        <f>'TOTAL RH'!D19</f>
+        <v/>
+      </c>
       <c r="E27" s="1" t="n"/>
       <c r="F27" s="1" t="n"/>
       <c r="G27" s="1" t="n"/>
-      <c r="H27" s="46">
-        <f>'TOTAL RH'!H3</f>
-        <v/>
-      </c>
-      <c r="I27" s="62" t="n"/>
-      <c r="J27" s="63" t="n"/>
+      <c r="H27" s="24" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="I27" s="51">
+        <f>'TOTAL RH'!I19</f>
+        <v/>
+      </c>
+      <c r="J27" s="51">
+        <f>'TOTAL RH'!J19</f>
+        <v/>
+      </c>
       <c r="K27" s="1" t="n"/>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n"/>
@@ -13413,31 +13340,15 @@
     </row>
     <row r="28" ht="13" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="24" t="n"/>
-      <c r="C28" s="47" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="D28" s="47" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="n"/>
+      <c r="D28" s="1" t="n"/>
       <c r="E28" s="1" t="n"/>
       <c r="F28" s="1" t="n"/>
       <c r="G28" s="1" t="n"/>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="47" t="inlineStr">
-        <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="J28" s="47" t="inlineStr">
-        <is>
-          <t>40'RH</t>
-        </is>
-      </c>
+      <c r="H28" s="1" t="n"/>
+      <c r="I28" s="1" t="n"/>
+      <c r="J28" s="1" t="n"/>
       <c r="K28" s="1" t="n"/>
       <c r="L28" s="1" t="n"/>
       <c r="M28" s="1" t="n"/>
@@ -13447,35 +13358,15 @@
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="1" t="n"/>
-      <c r="B29" s="24" t="inlineStr">
-        <is>
-          <t>AV</t>
-        </is>
-      </c>
-      <c r="C29" s="51">
-        <f>'TOTAL RH'!C21</f>
-        <v/>
-      </c>
-      <c r="D29" s="51">
-        <f>'TOTAL RH'!D21</f>
-        <v/>
-      </c>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
+      <c r="D29" s="1" t="n"/>
       <c r="E29" s="1" t="n"/>
       <c r="F29" s="1" t="n"/>
       <c r="G29" s="1" t="n"/>
-      <c r="H29" s="24" t="inlineStr">
-        <is>
-          <t>AV</t>
-        </is>
-      </c>
-      <c r="I29" s="51">
-        <f>'TOTAL RH'!I21</f>
-        <v/>
-      </c>
-      <c r="J29" s="51">
-        <f>'TOTAL RH'!J21</f>
-        <v/>
-      </c>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
       <c r="K29" s="1" t="n"/>
       <c r="L29" s="1" t="n"/>
       <c r="M29" s="1" t="n"/>
@@ -13485,35 +13376,19 @@
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="1" t="n"/>
-      <c r="B30" s="24" t="inlineStr">
-        <is>
-          <t>DMG</t>
-        </is>
-      </c>
-      <c r="C30" s="51">
-        <f>'TOTAL RH'!C22</f>
-        <v/>
-      </c>
-      <c r="D30" s="51">
-        <f>'TOTAL RH'!D22</f>
-        <v/>
-      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>RF SEASONAL — build year</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="n"/>
+      <c r="D30" s="1" t="n"/>
       <c r="E30" s="1" t="n"/>
       <c r="F30" s="1" t="n"/>
       <c r="G30" s="1" t="n"/>
-      <c r="H30" s="24" t="inlineStr">
-        <is>
-          <t>DMG</t>
-        </is>
-      </c>
-      <c r="I30" s="51">
-        <f>'TOTAL RH'!I22</f>
-        <v/>
-      </c>
-      <c r="J30" s="51">
-        <f>'TOTAL RH'!J22</f>
-        <v/>
-      </c>
+      <c r="H30" s="1" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="1" t="n"/>
       <c r="K30" s="1" t="n"/>
       <c r="L30" s="1" t="n"/>
       <c r="M30" s="1" t="n"/>
@@ -13523,17 +13398,29 @@
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="1" t="n"/>
-      <c r="B31" s="1" t="n"/>
-      <c r="C31" s="1" t="n"/>
-      <c r="D31" s="1" t="n"/>
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>BKK27 2020-26 BUILT</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
       <c r="E31" s="1" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="1" t="n"/>
+      <c r="F31" s="40" t="inlineStr">
+        <is>
+          <t>LCH27 2020-26 BUILT</t>
+        </is>
+      </c>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
       <c r="I31" s="1" t="n"/>
-      <c r="J31" s="1" t="n"/>
-      <c r="K31" s="1" t="n"/>
-      <c r="L31" s="1" t="n"/>
+      <c r="J31" s="40" t="inlineStr">
+        <is>
+          <t>PEAK BUILD YEAR</t>
+        </is>
+      </c>
+      <c r="K31" s="24" t="n"/>
+      <c r="L31" s="24" t="n"/>
       <c r="M31" s="1" t="n"/>
       <c r="N31" s="1" t="n"/>
       <c r="O31" s="1" t="n"/>
@@ -13541,17 +13428,26 @@
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" s="1" t="n"/>
-      <c r="B32" s="1" t="n"/>
-      <c r="C32" s="1" t="n"/>
-      <c r="D32" s="1" t="n"/>
+      <c r="B32" s="54">
+        <f>SUM('YEAR BUILT'!D11:D17)+SUM('YEAR BUILT'!F11:F17)+SUM('YEAR BUILT'!H11:H17)</f>
+        <v/>
+      </c>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
       <c r="E32" s="1" t="n"/>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="1" t="n"/>
-      <c r="H32" s="1" t="n"/>
+      <c r="F32" s="55">
+        <f>SUM('YEAR BUILT'!L11:L17)+SUM('YEAR BUILT'!N11:N17)+SUM('YEAR BUILT'!P11:P17)</f>
+        <v/>
+      </c>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
       <c r="I32" s="1" t="n"/>
-      <c r="J32" s="1" t="n"/>
-      <c r="K32" s="1" t="n"/>
-      <c r="L32" s="1" t="n"/>
+      <c r="J32" s="42">
+        <f>"2025"</f>
+        <v/>
+      </c>
+      <c r="K32" s="24" t="n"/>
+      <c r="L32" s="24" t="n"/>
       <c r="M32" s="1" t="n"/>
       <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
@@ -13559,21 +13455,29 @@
     </row>
     <row r="33" ht="13" customHeight="1">
       <c r="A33" s="1" t="n"/>
-      <c r="B33" s="44" t="inlineStr">
-        <is>
-          <t>RF SEASONAL — build year</t>
-        </is>
-      </c>
-      <c r="C33" s="1" t="n"/>
-      <c r="D33" s="1" t="n"/>
+      <c r="B33" s="43" t="inlineStr">
+        <is>
+          <t>of 40'RH on hand</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
       <c r="E33" s="1" t="n"/>
-      <c r="F33" s="1" t="n"/>
-      <c r="G33" s="1" t="n"/>
-      <c r="H33" s="1" t="n"/>
+      <c r="F33" s="43" t="inlineStr">
+        <is>
+          <t>of 40'RH on hand</t>
+        </is>
+      </c>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
       <c r="I33" s="1" t="n"/>
-      <c r="J33" s="1" t="n"/>
-      <c r="K33" s="1" t="n"/>
-      <c r="L33" s="1" t="n"/>
+      <c r="J33" s="43" t="inlineStr">
+        <is>
+          <t>13 units across both depots</t>
+        </is>
+      </c>
+      <c r="K33" s="24" t="n"/>
+      <c r="L33" s="24" t="n"/>
       <c r="M33" s="1" t="n"/>
       <c r="N33" s="1" t="n"/>
       <c r="O33" s="1" t="n"/>
@@ -13581,29 +13485,17 @@
     </row>
     <row r="34" ht="13" customHeight="1">
       <c r="A34" s="1" t="n"/>
-      <c r="B34" s="40" t="inlineStr">
-        <is>
-          <t>BKK27 2020-26 BUILT</t>
-        </is>
-      </c>
-      <c r="C34" s="24" t="n"/>
-      <c r="D34" s="24" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="n"/>
       <c r="E34" s="1" t="n"/>
-      <c r="F34" s="40" t="inlineStr">
-        <is>
-          <t>LCH27 2020-26 BUILT</t>
-        </is>
-      </c>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="n"/>
+      <c r="H34" s="1" t="n"/>
       <c r="I34" s="1" t="n"/>
-      <c r="J34" s="40" t="inlineStr">
-        <is>
-          <t>PEAK BUILD YEAR</t>
-        </is>
-      </c>
-      <c r="K34" s="24" t="n"/>
-      <c r="L34" s="24" t="n"/>
+      <c r="J34" s="1" t="n"/>
+      <c r="K34" s="1" t="n"/>
+      <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n"/>
       <c r="N34" s="1" t="n"/>
       <c r="O34" s="1" t="n"/>
@@ -13611,188 +13503,211 @@
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
-      <c r="B35" s="54">
-        <f>SUM('YEAR BUILT'!D11:D17)+SUM('YEAR BUILT'!F11:F17)+SUM('YEAR BUILT'!H11:H17)</f>
-        <v/>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>BKK27 DURIAN  (2021-2026)</t>
+        </is>
       </c>
       <c r="C35" s="24" t="n"/>
       <c r="D35" s="24" t="n"/>
       <c r="E35" s="1" t="n"/>
-      <c r="F35" s="55">
-        <f>SUM('YEAR BUILT'!L11:L17)+SUM('YEAR BUILT'!N11:N17)+SUM('YEAR BUILT'!P11:P17)</f>
-        <v/>
+      <c r="F35" s="40" t="inlineStr">
+        <is>
+          <t>BKK27 NON DURIAN  (≤ 2020)</t>
+        </is>
       </c>
       <c r="G35" s="24" t="n"/>
       <c r="H35" s="24" t="n"/>
       <c r="I35" s="1" t="n"/>
-      <c r="J35" s="42">
-        <f>"2025"</f>
-        <v/>
+      <c r="J35" s="40" t="inlineStr">
+        <is>
+          <t>LCH27 DURIAN  (2021-2026)</t>
+        </is>
       </c>
       <c r="K35" s="24" t="n"/>
       <c r="L35" s="24" t="n"/>
       <c r="M35" s="1" t="n"/>
-      <c r="N35" s="1" t="n"/>
-      <c r="O35" s="1" t="n"/>
-      <c r="P35" s="1" t="n"/>
+      <c r="N35" s="40" t="inlineStr">
+        <is>
+          <t>LCH27 NON DURIAN  (≤ 2020)</t>
+        </is>
+      </c>
+      <c r="O35" s="24" t="n"/>
+      <c r="P35" s="24" t="n"/>
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="1" t="n"/>
-      <c r="B36" s="43" t="inlineStr">
-        <is>
-          <t>of 40'RH on hand</t>
-        </is>
+      <c r="B36" s="54">
+        <f>'YEAR BUILT'!B4</f>
+        <v/>
       </c>
       <c r="C36" s="24" t="n"/>
       <c r="D36" s="24" t="n"/>
       <c r="E36" s="1" t="n"/>
-      <c r="F36" s="43" t="inlineStr">
-        <is>
-          <t>of 40'RH on hand</t>
-        </is>
+      <c r="F36" s="54">
+        <f>'YEAR BUILT'!F4</f>
+        <v/>
       </c>
       <c r="G36" s="24" t="n"/>
       <c r="H36" s="24" t="n"/>
       <c r="I36" s="1" t="n"/>
-      <c r="J36" s="43" t="inlineStr">
-        <is>
-          <t>13 units across both depots</t>
-        </is>
+      <c r="J36" s="55">
+        <f>'YEAR BUILT'!J4</f>
+        <v/>
       </c>
       <c r="K36" s="24" t="n"/>
       <c r="L36" s="24" t="n"/>
       <c r="M36" s="1" t="n"/>
-      <c r="N36" s="1" t="n"/>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
+      <c r="N36" s="55">
+        <f>'YEAR BUILT'!N4</f>
+        <v/>
+      </c>
+      <c r="O36" s="24" t="n"/>
+      <c r="P36" s="24" t="n"/>
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="1" t="n"/>
-      <c r="D37" s="1" t="n"/>
+      <c r="B37" s="43" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
       <c r="E37" s="1" t="n"/>
-      <c r="F37" s="1" t="n"/>
-      <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
+      <c r="F37" s="43" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
       <c r="I37" s="1" t="n"/>
-      <c r="J37" s="1" t="n"/>
-      <c r="K37" s="1" t="n"/>
-      <c r="L37" s="1" t="n"/>
+      <c r="J37" s="43" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="K37" s="24" t="n"/>
+      <c r="L37" s="24" t="n"/>
       <c r="M37" s="1" t="n"/>
-      <c r="N37" s="1" t="n"/>
-      <c r="O37" s="1" t="n"/>
-      <c r="P37" s="1" t="n"/>
+      <c r="N37" s="43" t="inlineStr">
+        <is>
+          <t>40'RH stock</t>
+        </is>
+      </c>
+      <c r="O37" s="24" t="n"/>
+      <c r="P37" s="24" t="n"/>
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" s="1" t="n"/>
-      <c r="B38" s="40" t="inlineStr">
-        <is>
-          <t>BKK27 DURIAN  (2021-2026)</t>
-        </is>
-      </c>
-      <c r="C38" s="24" t="n"/>
-      <c r="D38" s="24" t="n"/>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
       <c r="E38" s="1" t="n"/>
-      <c r="F38" s="40" t="inlineStr">
-        <is>
-          <t>BKK27 NON DURIAN  (≤ 2020)</t>
-        </is>
-      </c>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="24" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
       <c r="I38" s="1" t="n"/>
-      <c r="J38" s="40" t="inlineStr">
-        <is>
-          <t>LCH27 DURIAN  (2021-2026)</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="n"/>
-      <c r="L38" s="24" t="n"/>
+      <c r="J38" s="1" t="n"/>
+      <c r="K38" s="1" t="n"/>
+      <c r="L38" s="1" t="n"/>
       <c r="M38" s="1" t="n"/>
-      <c r="N38" s="40" t="inlineStr">
-        <is>
-          <t>LCH27 NON DURIAN  (≤ 2020)</t>
-        </is>
-      </c>
-      <c r="O38" s="24" t="n"/>
-      <c r="P38" s="24" t="n"/>
+      <c r="N38" s="1" t="n"/>
+      <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="n"/>
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="1" t="n"/>
-      <c r="B39" s="54">
-        <f>'YEAR BUILT'!B4</f>
-        <v/>
-      </c>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="24" t="n"/>
+      <c r="B39" s="45" t="inlineStr">
+        <is>
+          <t>BKK27 current mix</t>
+        </is>
+      </c>
+      <c r="C39" s="62" t="n"/>
+      <c r="D39" s="63" t="n"/>
       <c r="E39" s="1" t="n"/>
-      <c r="F39" s="54">
-        <f>'YEAR BUILT'!F4</f>
-        <v/>
-      </c>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="55">
-        <f>'YEAR BUILT'!J4</f>
-        <v/>
-      </c>
-      <c r="K39" s="24" t="n"/>
-      <c r="L39" s="24" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="46" t="inlineStr">
+        <is>
+          <t>LCH27 current mix</t>
+        </is>
+      </c>
+      <c r="I39" s="62" t="n"/>
+      <c r="J39" s="63" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
       <c r="M39" s="1" t="n"/>
-      <c r="N39" s="55">
-        <f>'YEAR BUILT'!N4</f>
-        <v/>
-      </c>
-      <c r="O39" s="24" t="n"/>
-      <c r="P39" s="24" t="n"/>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" s="1" t="n"/>
-      <c r="B40" s="43" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="C40" s="24" t="n"/>
-      <c r="D40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="47" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="D40" s="47" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
       <c r="E40" s="1" t="n"/>
-      <c r="F40" s="43" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="G40" s="24" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
       <c r="H40" s="24" t="n"/>
-      <c r="I40" s="1" t="n"/>
-      <c r="J40" s="43" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="K40" s="24" t="n"/>
-      <c r="L40" s="24" t="n"/>
+      <c r="I40" s="47" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="J40" s="47" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="n"/>
+      <c r="L40" s="1" t="n"/>
       <c r="M40" s="1" t="n"/>
-      <c r="N40" s="43" t="inlineStr">
-        <is>
-          <t>40'RH stock</t>
-        </is>
-      </c>
-      <c r="O40" s="24" t="n"/>
-      <c r="P40" s="24" t="n"/>
+      <c r="N40" s="1" t="n"/>
+      <c r="O40" s="1" t="n"/>
+      <c r="P40" s="1" t="n"/>
     </row>
     <row r="41" ht="13" customHeight="1">
       <c r="A41" s="1" t="n"/>
-      <c r="B41" s="1" t="n"/>
-      <c r="C41" s="1" t="n"/>
-      <c r="D41" s="1" t="n"/>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="C41" s="51">
+        <f>'YEAR BUILT'!C28</f>
+        <v/>
+      </c>
+      <c r="D41" s="51">
+        <f>'YEAR BUILT'!D28</f>
+        <v/>
+      </c>
       <c r="E41" s="1" t="n"/>
       <c r="F41" s="1" t="n"/>
       <c r="G41" s="1" t="n"/>
-      <c r="H41" s="1" t="n"/>
-      <c r="I41" s="1" t="n"/>
-      <c r="J41" s="1" t="n"/>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="I41" s="51">
+        <f>'YEAR BUILT'!K28</f>
+        <v/>
+      </c>
+      <c r="J41" s="51">
+        <f>'YEAR BUILT'!L28</f>
+        <v/>
+      </c>
       <c r="K41" s="1" t="n"/>
       <c r="L41" s="1" t="n"/>
       <c r="M41" s="1" t="n"/>
@@ -13802,23 +13717,35 @@
     </row>
     <row r="42" ht="13" customHeight="1">
       <c r="A42" s="1" t="n"/>
-      <c r="B42" s="45" t="inlineStr">
-        <is>
-          <t>BKK27 current mix</t>
-        </is>
-      </c>
-      <c r="C42" s="62" t="n"/>
-      <c r="D42" s="63" t="n"/>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="C42" s="51">
+        <f>'YEAR BUILT'!E28</f>
+        <v/>
+      </c>
+      <c r="D42" s="51">
+        <f>'YEAR BUILT'!F28</f>
+        <v/>
+      </c>
       <c r="E42" s="1" t="n"/>
       <c r="F42" s="1" t="n"/>
       <c r="G42" s="1" t="n"/>
-      <c r="H42" s="46" t="inlineStr">
-        <is>
-          <t>LCH27 current mix</t>
-        </is>
-      </c>
-      <c r="I42" s="62" t="n"/>
-      <c r="J42" s="63" t="n"/>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="I42" s="51">
+        <f>'YEAR BUILT'!M28</f>
+        <v/>
+      </c>
+      <c r="J42" s="51">
+        <f>'YEAR BUILT'!N28</f>
+        <v/>
+      </c>
       <c r="K42" s="1" t="n"/>
       <c r="L42" s="1" t="n"/>
       <c r="M42" s="1" t="n"/>
@@ -13828,30 +13755,34 @@
     </row>
     <row r="43" ht="13" customHeight="1">
       <c r="A43" s="1" t="n"/>
-      <c r="B43" s="24" t="n"/>
-      <c r="C43" s="47" t="inlineStr">
-        <is>
-          <t>22RE</t>
-        </is>
-      </c>
-      <c r="D43" s="47" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="C43" s="51">
+        <f>'YEAR BUILT'!G28</f>
+        <v/>
+      </c>
+      <c r="D43" s="51">
+        <f>'YEAR BUILT'!H28</f>
+        <v/>
       </c>
       <c r="E43" s="1" t="n"/>
       <c r="F43" s="1" t="n"/>
       <c r="G43" s="1" t="n"/>
-      <c r="H43" s="24" t="n"/>
-      <c r="I43" s="47" t="inlineStr">
-        <is>
-          <t>22RE</t>
-        </is>
-      </c>
-      <c r="J43" s="47" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
+      <c r="H43" s="24" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="I43" s="51">
+        <f>'YEAR BUILT'!O28</f>
+        <v/>
+      </c>
+      <c r="J43" s="51">
+        <f>'YEAR BUILT'!P28</f>
+        <v/>
       </c>
       <c r="K43" s="1" t="n"/>
       <c r="L43" s="1" t="n"/>
@@ -13862,35 +13793,15 @@
     </row>
     <row r="44" ht="13" customHeight="1">
       <c r="A44" s="1" t="n"/>
-      <c r="B44" s="24" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="C44" s="51">
-        <f>'YEAR BUILT'!C28</f>
-        <v/>
-      </c>
-      <c r="D44" s="51">
-        <f>'YEAR BUILT'!D28</f>
-        <v/>
-      </c>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
       <c r="E44" s="1" t="n"/>
       <c r="F44" s="1" t="n"/>
       <c r="G44" s="1" t="n"/>
-      <c r="H44" s="24" t="inlineStr">
-        <is>
-          <t>CARRIER</t>
-        </is>
-      </c>
-      <c r="I44" s="51">
-        <f>'YEAR BUILT'!K28</f>
-        <v/>
-      </c>
-      <c r="J44" s="51">
-        <f>'YEAR BUILT'!L28</f>
-        <v/>
-      </c>
+      <c r="H44" s="1" t="n"/>
+      <c r="I44" s="1" t="n"/>
+      <c r="J44" s="1" t="n"/>
       <c r="K44" s="1" t="n"/>
       <c r="L44" s="1" t="n"/>
       <c r="M44" s="1" t="n"/>
@@ -13900,35 +13811,19 @@
     </row>
     <row r="45" ht="13" customHeight="1">
       <c r="A45" s="1" t="n"/>
-      <c r="B45" s="24" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="C45" s="51">
-        <f>'YEAR BUILT'!E28</f>
-        <v/>
-      </c>
-      <c r="D45" s="51">
-        <f>'YEAR BUILT'!F28</f>
-        <v/>
-      </c>
+      <c r="B45" s="56" t="inlineStr">
+        <is>
+          <t>Full 2010-2026 Year x Brand x Size breakdown is on the YEAR BUILT sheet.</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="n"/>
+      <c r="D45" s="1" t="n"/>
       <c r="E45" s="1" t="n"/>
       <c r="F45" s="1" t="n"/>
       <c r="G45" s="1" t="n"/>
-      <c r="H45" s="24" t="inlineStr">
-        <is>
-          <t>DAIKIN</t>
-        </is>
-      </c>
-      <c r="I45" s="51">
-        <f>'YEAR BUILT'!M28</f>
-        <v/>
-      </c>
-      <c r="J45" s="51">
-        <f>'YEAR BUILT'!N28</f>
-        <v/>
-      </c>
+      <c r="H45" s="1" t="n"/>
+      <c r="I45" s="1" t="n"/>
+      <c r="J45" s="1" t="n"/>
       <c r="K45" s="1" t="n"/>
       <c r="L45" s="1" t="n"/>
       <c r="M45" s="1" t="n"/>
@@ -13936,93 +13831,15 @@
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="n"/>
     </row>
-    <row r="46" ht="13" customHeight="1">
-      <c r="A46" s="1" t="n"/>
-      <c r="B46" s="24" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="C46" s="51">
-        <f>'YEAR BUILT'!G28</f>
-        <v/>
-      </c>
-      <c r="D46" s="51">
-        <f>'YEAR BUILT'!H28</f>
-        <v/>
-      </c>
-      <c r="E46" s="1" t="n"/>
-      <c r="F46" s="1" t="n"/>
-      <c r="G46" s="1" t="n"/>
-      <c r="H46" s="24" t="inlineStr">
-        <is>
-          <t>THERMO KING</t>
-        </is>
-      </c>
-      <c r="I46" s="51">
-        <f>'YEAR BUILT'!O28</f>
-        <v/>
-      </c>
-      <c r="J46" s="51">
-        <f>'YEAR BUILT'!P28</f>
-        <v/>
-      </c>
-      <c r="K46" s="1" t="n"/>
-      <c r="L46" s="1" t="n"/>
-      <c r="M46" s="1" t="n"/>
-      <c r="N46" s="1" t="n"/>
-      <c r="O46" s="1" t="n"/>
-      <c r="P46" s="1" t="n"/>
-    </row>
-    <row r="47" ht="13" customHeight="1">
-      <c r="A47" s="1" t="n"/>
-      <c r="B47" s="1" t="n"/>
-      <c r="C47" s="1" t="n"/>
-      <c r="D47" s="1" t="n"/>
-      <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="n"/>
-      <c r="G47" s="1" t="n"/>
-      <c r="H47" s="1" t="n"/>
-      <c r="I47" s="1" t="n"/>
-      <c r="J47" s="1" t="n"/>
-      <c r="K47" s="1" t="n"/>
-      <c r="L47" s="1" t="n"/>
-      <c r="M47" s="1" t="n"/>
-      <c r="N47" s="1" t="n"/>
-      <c r="O47" s="1" t="n"/>
-      <c r="P47" s="1" t="n"/>
-    </row>
-    <row r="48" ht="13" customHeight="1">
-      <c r="A48" s="1" t="n"/>
-      <c r="B48" s="56" t="inlineStr">
-        <is>
-          <t>Full 2010-2026 Year x Brand x Size breakdown is on the YEAR BUILT sheet.</t>
-        </is>
-      </c>
-      <c r="C48" s="1" t="n"/>
-      <c r="D48" s="1" t="n"/>
-      <c r="E48" s="1" t="n"/>
-      <c r="F48" s="1" t="n"/>
-      <c r="G48" s="1" t="n"/>
-      <c r="H48" s="1" t="n"/>
-      <c r="I48" s="1" t="n"/>
-      <c r="J48" s="1" t="n"/>
-      <c r="K48" s="1" t="n"/>
-      <c r="L48" s="1" t="n"/>
-      <c r="M48" s="1" t="n"/>
-      <c r="N48" s="1" t="n"/>
-      <c r="O48" s="1" t="n"/>
-      <c r="P48" s="1" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="H24:J24"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B1:L2"/>
-    <mergeCell ref="B27:D27"/>
     <mergeCell ref="H9:J9"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="B24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>